<commit_message>
fixed small error in raw data that caused miscounting of CC abilities per character
</commit_message>
<xml_diff>
--- a/MRCC.xlsx
+++ b/MRCC.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mosta\Desktop\Projects\MarvelRivalsCC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1425765F-67D3-4BAA-A9DA-E9E3959E61D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CE58978-3F26-463C-AC97-9CCEAD842916}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" xr2:uid="{31EF6FEC-9292-46C9-88D6-31BB1C8D2748}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1461" uniqueCount="432">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1461" uniqueCount="431">
   <si>
     <t>Role</t>
   </si>
@@ -771,9 +771,6 @@
   </si>
   <si>
     <t>Flaming Meteor</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Y</t>
   </si>
   <si>
     <t>Blazing Blast</t>
@@ -1787,13 +1784,13 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>4</v>
@@ -1802,7 +1799,7 @@
         <v>5</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>111</v>
@@ -1811,7 +1808,7 @@
         <v>6</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>7</v>
@@ -1820,7 +1817,7 @@
         <v>8</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="P1" s="2" t="s">
         <v>9</v>
@@ -1829,7 +1826,7 @@
         <v>10</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="S1" s="2" t="s">
         <v>11</v>
@@ -1838,7 +1835,7 @@
         <v>12</v>
       </c>
       <c r="U1" s="2" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="V1" s="2" t="s">
         <v>13</v>
@@ -1847,7 +1844,7 @@
         <v>14</v>
       </c>
       <c r="X1" s="2" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="Y1" s="2" t="s">
         <v>15</v>
@@ -1856,7 +1853,7 @@
         <v>16</v>
       </c>
       <c r="AA1" s="2" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="AB1" s="2" t="s">
         <v>17</v>
@@ -1945,7 +1942,7 @@
         <v>96</v>
       </c>
       <c r="AB2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.3">
@@ -3833,22 +3830,22 @@
         <v>243</v>
       </c>
       <c r="T25" t="s">
-        <v>244</v>
+        <v>74</v>
       </c>
       <c r="U25" t="s">
         <v>98</v>
       </c>
       <c r="V25" t="s">
+        <v>244</v>
+      </c>
+      <c r="W25" t="s">
+        <v>75</v>
+      </c>
+      <c r="X25" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y25" t="s">
         <v>245</v>
-      </c>
-      <c r="W25" t="s">
-        <v>75</v>
-      </c>
-      <c r="X25" t="s">
-        <v>76</v>
-      </c>
-      <c r="Y25" t="s">
-        <v>246</v>
       </c>
       <c r="Z25" t="s">
         <v>75</v>
@@ -3877,7 +3874,7 @@
         <v>76</v>
       </c>
       <c r="G26" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="H26" t="s">
         <v>74</v>
@@ -3886,16 +3883,16 @@
         <v>98</v>
       </c>
       <c r="J26" t="s">
+        <v>247</v>
+      </c>
+      <c r="K26" t="s">
+        <v>75</v>
+      </c>
+      <c r="L26" t="s">
+        <v>76</v>
+      </c>
+      <c r="M26" t="s">
         <v>248</v>
-      </c>
-      <c r="K26" t="s">
-        <v>75</v>
-      </c>
-      <c r="L26" t="s">
-        <v>76</v>
-      </c>
-      <c r="M26" t="s">
-        <v>249</v>
       </c>
       <c r="N26" t="s">
         <v>74</v>
@@ -3904,34 +3901,34 @@
         <v>98</v>
       </c>
       <c r="P26" t="s">
+        <v>249</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>75</v>
+      </c>
+      <c r="R26" t="s">
+        <v>76</v>
+      </c>
+      <c r="S26" t="s">
         <v>250</v>
       </c>
-      <c r="Q26" t="s">
-        <v>75</v>
-      </c>
-      <c r="R26" t="s">
-        <v>76</v>
-      </c>
-      <c r="S26" t="s">
+      <c r="T26" t="s">
+        <v>75</v>
+      </c>
+      <c r="U26" t="s">
+        <v>76</v>
+      </c>
+      <c r="V26" t="s">
+        <v>76</v>
+      </c>
+      <c r="W26" t="s">
+        <v>76</v>
+      </c>
+      <c r="X26" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y26" t="s">
         <v>251</v>
-      </c>
-      <c r="T26" t="s">
-        <v>75</v>
-      </c>
-      <c r="U26" t="s">
-        <v>76</v>
-      </c>
-      <c r="V26" t="s">
-        <v>76</v>
-      </c>
-      <c r="W26" t="s">
-        <v>76</v>
-      </c>
-      <c r="X26" t="s">
-        <v>76</v>
-      </c>
-      <c r="Y26" t="s">
-        <v>252</v>
       </c>
       <c r="Z26" t="s">
         <v>75</v>
@@ -3960,61 +3957,61 @@
         <v>76</v>
       </c>
       <c r="G27" t="s">
+        <v>252</v>
+      </c>
+      <c r="H27" t="s">
+        <v>75</v>
+      </c>
+      <c r="I27" t="s">
+        <v>76</v>
+      </c>
+      <c r="J27" t="s">
         <v>253</v>
       </c>
-      <c r="H27" t="s">
-        <v>75</v>
-      </c>
-      <c r="I27" t="s">
-        <v>76</v>
-      </c>
-      <c r="J27" t="s">
+      <c r="K27" t="s">
+        <v>75</v>
+      </c>
+      <c r="L27" t="s">
+        <v>76</v>
+      </c>
+      <c r="M27" t="s">
         <v>254</v>
       </c>
-      <c r="K27" t="s">
-        <v>75</v>
-      </c>
-      <c r="L27" t="s">
-        <v>76</v>
-      </c>
-      <c r="M27" t="s">
+      <c r="N27" t="s">
+        <v>75</v>
+      </c>
+      <c r="O27" t="s">
+        <v>76</v>
+      </c>
+      <c r="P27" t="s">
         <v>255</v>
       </c>
-      <c r="N27" t="s">
-        <v>75</v>
-      </c>
-      <c r="O27" t="s">
-        <v>76</v>
-      </c>
-      <c r="P27" t="s">
+      <c r="Q27" t="s">
+        <v>75</v>
+      </c>
+      <c r="R27" t="s">
+        <v>76</v>
+      </c>
+      <c r="S27" t="s">
         <v>256</v>
       </c>
-      <c r="Q27" t="s">
-        <v>75</v>
-      </c>
-      <c r="R27" t="s">
-        <v>76</v>
-      </c>
-      <c r="S27" t="s">
+      <c r="T27" t="s">
+        <v>75</v>
+      </c>
+      <c r="U27" t="s">
+        <v>76</v>
+      </c>
+      <c r="V27" t="s">
+        <v>76</v>
+      </c>
+      <c r="W27" t="s">
+        <v>76</v>
+      </c>
+      <c r="X27" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y27" t="s">
         <v>257</v>
-      </c>
-      <c r="T27" t="s">
-        <v>75</v>
-      </c>
-      <c r="U27" t="s">
-        <v>76</v>
-      </c>
-      <c r="V27" t="s">
-        <v>76</v>
-      </c>
-      <c r="W27" t="s">
-        <v>76</v>
-      </c>
-      <c r="X27" t="s">
-        <v>76</v>
-      </c>
-      <c r="Y27" t="s">
-        <v>258</v>
       </c>
       <c r="Z27" t="s">
         <v>75</v>
@@ -4043,34 +4040,34 @@
         <v>76</v>
       </c>
       <c r="G28" t="s">
+        <v>258</v>
+      </c>
+      <c r="H28" t="s">
+        <v>75</v>
+      </c>
+      <c r="I28" t="s">
+        <v>76</v>
+      </c>
+      <c r="J28" t="s">
+        <v>261</v>
+      </c>
+      <c r="K28" t="s">
+        <v>75</v>
+      </c>
+      <c r="L28" t="s">
+        <v>76</v>
+      </c>
+      <c r="M28" t="s">
         <v>259</v>
       </c>
-      <c r="H28" t="s">
-        <v>75</v>
-      </c>
-      <c r="I28" t="s">
-        <v>76</v>
-      </c>
-      <c r="J28" t="s">
-        <v>262</v>
-      </c>
-      <c r="K28" t="s">
-        <v>75</v>
-      </c>
-      <c r="L28" t="s">
-        <v>76</v>
-      </c>
-      <c r="M28" t="s">
+      <c r="N28" t="s">
+        <v>75</v>
+      </c>
+      <c r="O28" t="s">
+        <v>76</v>
+      </c>
+      <c r="P28" t="s">
         <v>260</v>
-      </c>
-      <c r="N28" t="s">
-        <v>75</v>
-      </c>
-      <c r="O28" t="s">
-        <v>76</v>
-      </c>
-      <c r="P28" t="s">
-        <v>261</v>
       </c>
       <c r="Q28" t="s">
         <v>74</v>
@@ -4079,25 +4076,25 @@
         <v>92</v>
       </c>
       <c r="S28" t="s">
+        <v>262</v>
+      </c>
+      <c r="T28" t="s">
+        <v>75</v>
+      </c>
+      <c r="U28" t="s">
+        <v>76</v>
+      </c>
+      <c r="V28" t="s">
         <v>263</v>
       </c>
-      <c r="T28" t="s">
-        <v>75</v>
-      </c>
-      <c r="U28" t="s">
-        <v>76</v>
-      </c>
-      <c r="V28" t="s">
+      <c r="W28" t="s">
+        <v>75</v>
+      </c>
+      <c r="X28" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y28" t="s">
         <v>264</v>
-      </c>
-      <c r="W28" t="s">
-        <v>75</v>
-      </c>
-      <c r="X28" t="s">
-        <v>76</v>
-      </c>
-      <c r="Y28" t="s">
-        <v>265</v>
       </c>
       <c r="Z28" t="s">
         <v>75</v>
@@ -4126,34 +4123,34 @@
         <v>76</v>
       </c>
       <c r="G29" t="s">
+        <v>265</v>
+      </c>
+      <c r="H29" t="s">
+        <v>75</v>
+      </c>
+      <c r="I29" t="s">
+        <v>76</v>
+      </c>
+      <c r="J29" t="s">
         <v>266</v>
       </c>
-      <c r="H29" t="s">
-        <v>75</v>
-      </c>
-      <c r="I29" t="s">
-        <v>76</v>
-      </c>
-      <c r="J29" t="s">
+      <c r="K29" t="s">
+        <v>74</v>
+      </c>
+      <c r="L29" t="s">
         <v>267</v>
       </c>
-      <c r="K29" t="s">
-        <v>74</v>
-      </c>
-      <c r="L29" t="s">
+      <c r="M29" t="s">
         <v>268</v>
       </c>
-      <c r="M29" t="s">
+      <c r="N29" t="s">
+        <v>75</v>
+      </c>
+      <c r="O29" t="s">
+        <v>76</v>
+      </c>
+      <c r="P29" t="s">
         <v>269</v>
-      </c>
-      <c r="N29" t="s">
-        <v>75</v>
-      </c>
-      <c r="O29" t="s">
-        <v>76</v>
-      </c>
-      <c r="P29" t="s">
-        <v>270</v>
       </c>
       <c r="Q29" t="s">
         <v>74</v>
@@ -4180,7 +4177,7 @@
         <v>76</v>
       </c>
       <c r="Y29" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="Z29" t="s">
         <v>74</v>
@@ -4209,34 +4206,34 @@
         <v>98</v>
       </c>
       <c r="G30" t="s">
+        <v>271</v>
+      </c>
+      <c r="H30" t="s">
+        <v>75</v>
+      </c>
+      <c r="I30" t="s">
+        <v>76</v>
+      </c>
+      <c r="J30" t="s">
         <v>272</v>
       </c>
-      <c r="H30" t="s">
-        <v>75</v>
-      </c>
-      <c r="I30" t="s">
-        <v>76</v>
-      </c>
-      <c r="J30" t="s">
+      <c r="K30" t="s">
+        <v>75</v>
+      </c>
+      <c r="L30" t="s">
+        <v>76</v>
+      </c>
+      <c r="M30" t="s">
         <v>273</v>
       </c>
-      <c r="K30" t="s">
-        <v>75</v>
-      </c>
-      <c r="L30" t="s">
-        <v>76</v>
-      </c>
-      <c r="M30" t="s">
+      <c r="N30" t="s">
+        <v>75</v>
+      </c>
+      <c r="O30" t="s">
+        <v>76</v>
+      </c>
+      <c r="P30" t="s">
         <v>274</v>
-      </c>
-      <c r="N30" t="s">
-        <v>75</v>
-      </c>
-      <c r="O30" t="s">
-        <v>76</v>
-      </c>
-      <c r="P30" t="s">
-        <v>275</v>
       </c>
       <c r="Q30" t="s">
         <v>74</v>
@@ -4245,25 +4242,25 @@
         <v>97</v>
       </c>
       <c r="S30" t="s">
+        <v>275</v>
+      </c>
+      <c r="T30" t="s">
+        <v>75</v>
+      </c>
+      <c r="U30" t="s">
+        <v>76</v>
+      </c>
+      <c r="V30" t="s">
         <v>276</v>
       </c>
-      <c r="T30" t="s">
-        <v>75</v>
-      </c>
-      <c r="U30" t="s">
-        <v>76</v>
-      </c>
-      <c r="V30" t="s">
+      <c r="W30" t="s">
+        <v>75</v>
+      </c>
+      <c r="X30" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y30" t="s">
         <v>277</v>
-      </c>
-      <c r="W30" t="s">
-        <v>75</v>
-      </c>
-      <c r="X30" t="s">
-        <v>76</v>
-      </c>
-      <c r="Y30" t="s">
-        <v>278</v>
       </c>
       <c r="Z30" t="s">
         <v>75</v>
@@ -4292,67 +4289,67 @@
         <v>76</v>
       </c>
       <c r="G31" t="s">
+        <v>278</v>
+      </c>
+      <c r="H31" t="s">
+        <v>75</v>
+      </c>
+      <c r="I31" t="s">
+        <v>76</v>
+      </c>
+      <c r="J31" t="s">
         <v>279</v>
       </c>
-      <c r="H31" t="s">
-        <v>75</v>
-      </c>
-      <c r="I31" t="s">
-        <v>76</v>
-      </c>
-      <c r="J31" t="s">
+      <c r="K31" t="s">
+        <v>75</v>
+      </c>
+      <c r="L31" t="s">
+        <v>76</v>
+      </c>
+      <c r="M31" t="s">
         <v>280</v>
       </c>
-      <c r="K31" t="s">
-        <v>75</v>
-      </c>
-      <c r="L31" t="s">
-        <v>76</v>
-      </c>
-      <c r="M31" t="s">
+      <c r="N31" t="s">
+        <v>75</v>
+      </c>
+      <c r="O31" t="s">
+        <v>76</v>
+      </c>
+      <c r="P31" t="s">
         <v>281</v>
       </c>
-      <c r="N31" t="s">
-        <v>75</v>
-      </c>
-      <c r="O31" t="s">
-        <v>76</v>
-      </c>
-      <c r="P31" t="s">
+      <c r="Q31" t="s">
+        <v>75</v>
+      </c>
+      <c r="R31" t="s">
+        <v>76</v>
+      </c>
+      <c r="S31" t="s">
         <v>282</v>
       </c>
-      <c r="Q31" t="s">
-        <v>75</v>
-      </c>
-      <c r="R31" t="s">
-        <v>76</v>
-      </c>
-      <c r="S31" t="s">
+      <c r="T31" t="s">
+        <v>75</v>
+      </c>
+      <c r="U31" t="s">
+        <v>76</v>
+      </c>
+      <c r="V31" t="s">
+        <v>76</v>
+      </c>
+      <c r="W31" t="s">
+        <v>76</v>
+      </c>
+      <c r="X31" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y31" t="s">
         <v>283</v>
       </c>
-      <c r="T31" t="s">
-        <v>75</v>
-      </c>
-      <c r="U31" t="s">
-        <v>76</v>
-      </c>
-      <c r="V31" t="s">
-        <v>76</v>
-      </c>
-      <c r="W31" t="s">
-        <v>76</v>
-      </c>
-      <c r="X31" t="s">
-        <v>76</v>
-      </c>
-      <c r="Y31" t="s">
+      <c r="Z31" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA31" t="s">
         <v>284</v>
-      </c>
-      <c r="Z31" t="s">
-        <v>74</v>
-      </c>
-      <c r="AA31" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="32" spans="1:27" x14ac:dyDescent="0.3">
@@ -4375,61 +4372,61 @@
         <v>76</v>
       </c>
       <c r="G32" t="s">
+        <v>285</v>
+      </c>
+      <c r="H32" t="s">
+        <v>75</v>
+      </c>
+      <c r="I32" t="s">
+        <v>76</v>
+      </c>
+      <c r="J32" t="s">
         <v>286</v>
       </c>
-      <c r="H32" t="s">
-        <v>75</v>
-      </c>
-      <c r="I32" t="s">
-        <v>76</v>
-      </c>
-      <c r="J32" t="s">
+      <c r="K32" t="s">
+        <v>74</v>
+      </c>
+      <c r="L32" t="s">
         <v>287</v>
       </c>
-      <c r="K32" t="s">
-        <v>75</v>
-      </c>
-      <c r="L32" t="s">
+      <c r="M32" t="s">
         <v>288</v>
       </c>
-      <c r="M32" t="s">
+      <c r="N32" t="s">
+        <v>75</v>
+      </c>
+      <c r="O32" t="s">
+        <v>76</v>
+      </c>
+      <c r="P32" t="s">
         <v>289</v>
       </c>
-      <c r="N32" t="s">
-        <v>75</v>
-      </c>
-      <c r="O32" t="s">
-        <v>76</v>
-      </c>
-      <c r="P32" t="s">
+      <c r="Q32" t="s">
+        <v>75</v>
+      </c>
+      <c r="R32" t="s">
+        <v>76</v>
+      </c>
+      <c r="S32" t="s">
+        <v>76</v>
+      </c>
+      <c r="T32" t="s">
+        <v>76</v>
+      </c>
+      <c r="U32" t="s">
+        <v>76</v>
+      </c>
+      <c r="V32" t="s">
+        <v>76</v>
+      </c>
+      <c r="W32" t="s">
+        <v>76</v>
+      </c>
+      <c r="X32" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y32" t="s">
         <v>290</v>
-      </c>
-      <c r="Q32" t="s">
-        <v>75</v>
-      </c>
-      <c r="R32" t="s">
-        <v>76</v>
-      </c>
-      <c r="S32" t="s">
-        <v>76</v>
-      </c>
-      <c r="T32" t="s">
-        <v>76</v>
-      </c>
-      <c r="U32" t="s">
-        <v>76</v>
-      </c>
-      <c r="V32" t="s">
-        <v>76</v>
-      </c>
-      <c r="W32" t="s">
-        <v>76</v>
-      </c>
-      <c r="X32" t="s">
-        <v>76</v>
-      </c>
-      <c r="Y32" t="s">
-        <v>291</v>
       </c>
       <c r="Z32" t="s">
         <v>75</v>
@@ -4458,61 +4455,61 @@
         <v>76</v>
       </c>
       <c r="G33" t="s">
+        <v>291</v>
+      </c>
+      <c r="H33" t="s">
+        <v>75</v>
+      </c>
+      <c r="I33" t="s">
+        <v>76</v>
+      </c>
+      <c r="J33" t="s">
         <v>292</v>
       </c>
-      <c r="H33" t="s">
-        <v>75</v>
-      </c>
-      <c r="I33" t="s">
-        <v>76</v>
-      </c>
-      <c r="J33" t="s">
+      <c r="K33" t="s">
+        <v>75</v>
+      </c>
+      <c r="L33" t="s">
+        <v>76</v>
+      </c>
+      <c r="M33" t="s">
         <v>293</v>
       </c>
-      <c r="K33" t="s">
-        <v>75</v>
-      </c>
-      <c r="L33" t="s">
-        <v>76</v>
-      </c>
-      <c r="M33" t="s">
+      <c r="N33" t="s">
+        <v>75</v>
+      </c>
+      <c r="O33" t="s">
+        <v>76</v>
+      </c>
+      <c r="P33" t="s">
         <v>294</v>
       </c>
-      <c r="N33" t="s">
-        <v>75</v>
-      </c>
-      <c r="O33" t="s">
-        <v>76</v>
-      </c>
-      <c r="P33" t="s">
+      <c r="Q33" t="s">
+        <v>75</v>
+      </c>
+      <c r="R33" t="s">
+        <v>76</v>
+      </c>
+      <c r="S33" t="s">
+        <v>76</v>
+      </c>
+      <c r="T33" t="s">
+        <v>76</v>
+      </c>
+      <c r="U33" t="s">
+        <v>76</v>
+      </c>
+      <c r="V33" t="s">
+        <v>76</v>
+      </c>
+      <c r="W33" t="s">
+        <v>76</v>
+      </c>
+      <c r="X33" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y33" t="s">
         <v>295</v>
-      </c>
-      <c r="Q33" t="s">
-        <v>75</v>
-      </c>
-      <c r="R33" t="s">
-        <v>76</v>
-      </c>
-      <c r="S33" t="s">
-        <v>76</v>
-      </c>
-      <c r="T33" t="s">
-        <v>76</v>
-      </c>
-      <c r="U33" t="s">
-        <v>76</v>
-      </c>
-      <c r="V33" t="s">
-        <v>76</v>
-      </c>
-      <c r="W33" t="s">
-        <v>76</v>
-      </c>
-      <c r="X33" t="s">
-        <v>76</v>
-      </c>
-      <c r="Y33" t="s">
-        <v>296</v>
       </c>
       <c r="Z33" t="s">
         <v>75</v>
@@ -4541,34 +4538,34 @@
         <v>76</v>
       </c>
       <c r="G34" t="s">
+        <v>296</v>
+      </c>
+      <c r="H34" t="s">
+        <v>75</v>
+      </c>
+      <c r="I34" t="s">
+        <v>76</v>
+      </c>
+      <c r="J34" t="s">
         <v>297</v>
       </c>
-      <c r="H34" t="s">
-        <v>75</v>
-      </c>
-      <c r="I34" t="s">
-        <v>76</v>
-      </c>
-      <c r="J34" t="s">
+      <c r="K34" t="s">
+        <v>75</v>
+      </c>
+      <c r="L34" t="s">
+        <v>76</v>
+      </c>
+      <c r="M34" t="s">
         <v>298</v>
       </c>
-      <c r="K34" t="s">
-        <v>75</v>
-      </c>
-      <c r="L34" t="s">
-        <v>76</v>
-      </c>
-      <c r="M34" t="s">
+      <c r="N34" t="s">
+        <v>75</v>
+      </c>
+      <c r="O34" t="s">
+        <v>76</v>
+      </c>
+      <c r="P34" t="s">
         <v>299</v>
-      </c>
-      <c r="N34" t="s">
-        <v>75</v>
-      </c>
-      <c r="O34" t="s">
-        <v>76</v>
-      </c>
-      <c r="P34" t="s">
-        <v>300</v>
       </c>
       <c r="Q34" t="s">
         <v>74</v>
@@ -4577,7 +4574,7 @@
         <v>94</v>
       </c>
       <c r="S34" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="T34" t="s">
         <v>222</v>
@@ -4595,7 +4592,7 @@
         <v>76</v>
       </c>
       <c r="Y34" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="Z34" t="s">
         <v>74</v>
@@ -4624,34 +4621,34 @@
         <v>76</v>
       </c>
       <c r="G35" t="s">
+        <v>302</v>
+      </c>
+      <c r="H35" t="s">
+        <v>75</v>
+      </c>
+      <c r="I35" t="s">
+        <v>76</v>
+      </c>
+      <c r="J35" t="s">
         <v>303</v>
       </c>
-      <c r="H35" t="s">
-        <v>75</v>
-      </c>
-      <c r="I35" t="s">
-        <v>76</v>
-      </c>
-      <c r="J35" t="s">
+      <c r="K35" t="s">
+        <v>75</v>
+      </c>
+      <c r="L35" t="s">
+        <v>76</v>
+      </c>
+      <c r="M35" t="s">
         <v>304</v>
       </c>
-      <c r="K35" t="s">
-        <v>75</v>
-      </c>
-      <c r="L35" t="s">
-        <v>76</v>
-      </c>
-      <c r="M35" t="s">
+      <c r="N35" t="s">
+        <v>75</v>
+      </c>
+      <c r="O35" t="s">
+        <v>76</v>
+      </c>
+      <c r="P35" t="s">
         <v>305</v>
-      </c>
-      <c r="N35" t="s">
-        <v>75</v>
-      </c>
-      <c r="O35" t="s">
-        <v>76</v>
-      </c>
-      <c r="P35" t="s">
-        <v>306</v>
       </c>
       <c r="Q35" t="s">
         <v>74</v>
@@ -4660,7 +4657,7 @@
         <v>91</v>
       </c>
       <c r="S35" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="T35" t="s">
         <v>74</v>
@@ -4669,22 +4666,22 @@
         <v>92</v>
       </c>
       <c r="V35" t="s">
+        <v>307</v>
+      </c>
+      <c r="W35" t="s">
+        <v>75</v>
+      </c>
+      <c r="X35" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y35" t="s">
         <v>308</v>
       </c>
-      <c r="W35" t="s">
-        <v>75</v>
-      </c>
-      <c r="X35" t="s">
-        <v>76</v>
-      </c>
-      <c r="Y35" t="s">
+      <c r="Z35" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA35" t="s">
         <v>309</v>
-      </c>
-      <c r="Z35" t="s">
-        <v>74</v>
-      </c>
-      <c r="AA35" t="s">
-        <v>310</v>
       </c>
     </row>
     <row r="36" spans="1:28" x14ac:dyDescent="0.3">
@@ -4707,16 +4704,16 @@
         <v>76</v>
       </c>
       <c r="G36" t="s">
+        <v>310</v>
+      </c>
+      <c r="H36" t="s">
+        <v>75</v>
+      </c>
+      <c r="I36" t="s">
+        <v>76</v>
+      </c>
+      <c r="J36" t="s">
         <v>311</v>
-      </c>
-      <c r="H36" t="s">
-        <v>75</v>
-      </c>
-      <c r="I36" t="s">
-        <v>76</v>
-      </c>
-      <c r="J36" t="s">
-        <v>312</v>
       </c>
       <c r="K36" t="s">
         <v>74</v>
@@ -4725,43 +4722,43 @@
         <v>224</v>
       </c>
       <c r="M36" t="s">
+        <v>312</v>
+      </c>
+      <c r="N36" t="s">
+        <v>75</v>
+      </c>
+      <c r="O36" t="s">
+        <v>76</v>
+      </c>
+      <c r="P36" t="s">
         <v>313</v>
       </c>
-      <c r="N36" t="s">
-        <v>75</v>
-      </c>
-      <c r="O36" t="s">
-        <v>76</v>
-      </c>
-      <c r="P36" t="s">
+      <c r="Q36" t="s">
+        <v>75</v>
+      </c>
+      <c r="R36" t="s">
+        <v>76</v>
+      </c>
+      <c r="S36" t="s">
+        <v>76</v>
+      </c>
+      <c r="T36" t="s">
+        <v>76</v>
+      </c>
+      <c r="U36" t="s">
+        <v>76</v>
+      </c>
+      <c r="V36" t="s">
+        <v>76</v>
+      </c>
+      <c r="W36" t="s">
+        <v>76</v>
+      </c>
+      <c r="X36" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y36" t="s">
         <v>314</v>
-      </c>
-      <c r="Q36" t="s">
-        <v>75</v>
-      </c>
-      <c r="R36" t="s">
-        <v>76</v>
-      </c>
-      <c r="S36" t="s">
-        <v>76</v>
-      </c>
-      <c r="T36" t="s">
-        <v>76</v>
-      </c>
-      <c r="U36" t="s">
-        <v>76</v>
-      </c>
-      <c r="V36" t="s">
-        <v>76</v>
-      </c>
-      <c r="W36" t="s">
-        <v>76</v>
-      </c>
-      <c r="X36" t="s">
-        <v>76</v>
-      </c>
-      <c r="Y36" t="s">
-        <v>315</v>
       </c>
       <c r="Z36" t="s">
         <v>75</v>
@@ -4790,61 +4787,61 @@
         <v>76</v>
       </c>
       <c r="G37" t="s">
+        <v>315</v>
+      </c>
+      <c r="H37" t="s">
+        <v>75</v>
+      </c>
+      <c r="I37" t="s">
+        <v>76</v>
+      </c>
+      <c r="J37" t="s">
+        <v>76</v>
+      </c>
+      <c r="K37" t="s">
+        <v>76</v>
+      </c>
+      <c r="L37" t="s">
+        <v>76</v>
+      </c>
+      <c r="M37" t="s">
         <v>316</v>
       </c>
-      <c r="H37" t="s">
-        <v>75</v>
-      </c>
-      <c r="I37" t="s">
-        <v>76</v>
-      </c>
-      <c r="J37" t="s">
-        <v>76</v>
-      </c>
-      <c r="K37" t="s">
-        <v>76</v>
-      </c>
-      <c r="L37" t="s">
-        <v>76</v>
-      </c>
-      <c r="M37" t="s">
+      <c r="N37" t="s">
+        <v>75</v>
+      </c>
+      <c r="O37" t="s">
+        <v>76</v>
+      </c>
+      <c r="P37" t="s">
         <v>317</v>
       </c>
-      <c r="N37" t="s">
-        <v>75</v>
-      </c>
-      <c r="O37" t="s">
-        <v>76</v>
-      </c>
-      <c r="P37" t="s">
+      <c r="Q37" t="s">
+        <v>75</v>
+      </c>
+      <c r="R37" t="s">
+        <v>76</v>
+      </c>
+      <c r="S37" t="s">
         <v>318</v>
       </c>
-      <c r="Q37" t="s">
-        <v>75</v>
-      </c>
-      <c r="R37" t="s">
-        <v>76</v>
-      </c>
-      <c r="S37" t="s">
+      <c r="T37" t="s">
+        <v>75</v>
+      </c>
+      <c r="U37" t="s">
+        <v>76</v>
+      </c>
+      <c r="V37" t="s">
+        <v>76</v>
+      </c>
+      <c r="W37" t="s">
+        <v>76</v>
+      </c>
+      <c r="X37" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y37" t="s">
         <v>319</v>
-      </c>
-      <c r="T37" t="s">
-        <v>75</v>
-      </c>
-      <c r="U37" t="s">
-        <v>76</v>
-      </c>
-      <c r="V37" t="s">
-        <v>76</v>
-      </c>
-      <c r="W37" t="s">
-        <v>76</v>
-      </c>
-      <c r="X37" t="s">
-        <v>76</v>
-      </c>
-      <c r="Y37" t="s">
-        <v>320</v>
       </c>
       <c r="Z37" t="s">
         <v>75</v>
@@ -4873,34 +4870,34 @@
         <v>76</v>
       </c>
       <c r="G38" t="s">
+        <v>320</v>
+      </c>
+      <c r="H38" t="s">
+        <v>75</v>
+      </c>
+      <c r="I38" t="s">
+        <v>76</v>
+      </c>
+      <c r="J38" t="s">
+        <v>76</v>
+      </c>
+      <c r="K38" t="s">
+        <v>76</v>
+      </c>
+      <c r="L38" t="s">
+        <v>76</v>
+      </c>
+      <c r="M38" t="s">
         <v>321</v>
       </c>
-      <c r="H38" t="s">
-        <v>75</v>
-      </c>
-      <c r="I38" t="s">
-        <v>76</v>
-      </c>
-      <c r="J38" t="s">
-        <v>76</v>
-      </c>
-      <c r="K38" t="s">
-        <v>76</v>
-      </c>
-      <c r="L38" t="s">
-        <v>76</v>
-      </c>
-      <c r="M38" t="s">
+      <c r="N38" t="s">
+        <v>75</v>
+      </c>
+      <c r="O38" t="s">
+        <v>76</v>
+      </c>
+      <c r="P38" t="s">
         <v>322</v>
-      </c>
-      <c r="N38" t="s">
-        <v>75</v>
-      </c>
-      <c r="O38" t="s">
-        <v>76</v>
-      </c>
-      <c r="P38" t="s">
-        <v>323</v>
       </c>
       <c r="Q38" t="s">
         <v>74</v>
@@ -4909,25 +4906,25 @@
         <v>95</v>
       </c>
       <c r="S38" t="s">
+        <v>323</v>
+      </c>
+      <c r="T38" t="s">
+        <v>75</v>
+      </c>
+      <c r="U38" t="s">
+        <v>76</v>
+      </c>
+      <c r="V38" t="s">
+        <v>76</v>
+      </c>
+      <c r="W38" t="s">
+        <v>76</v>
+      </c>
+      <c r="X38" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y38" t="s">
         <v>324</v>
-      </c>
-      <c r="T38" t="s">
-        <v>75</v>
-      </c>
-      <c r="U38" t="s">
-        <v>76</v>
-      </c>
-      <c r="V38" t="s">
-        <v>76</v>
-      </c>
-      <c r="W38" t="s">
-        <v>76</v>
-      </c>
-      <c r="X38" t="s">
-        <v>76</v>
-      </c>
-      <c r="Y38" t="s">
-        <v>325</v>
       </c>
       <c r="Z38" t="s">
         <v>74</v>
@@ -4956,61 +4953,61 @@
         <v>76</v>
       </c>
       <c r="G39" t="s">
+        <v>325</v>
+      </c>
+      <c r="H39" t="s">
+        <v>75</v>
+      </c>
+      <c r="I39" t="s">
+        <v>76</v>
+      </c>
+      <c r="J39" t="s">
         <v>326</v>
       </c>
-      <c r="H39" t="s">
-        <v>75</v>
-      </c>
-      <c r="I39" t="s">
-        <v>76</v>
-      </c>
-      <c r="J39" t="s">
+      <c r="K39" t="s">
+        <v>75</v>
+      </c>
+      <c r="L39" t="s">
+        <v>76</v>
+      </c>
+      <c r="M39" t="s">
         <v>327</v>
       </c>
-      <c r="K39" t="s">
-        <v>75</v>
-      </c>
-      <c r="L39" t="s">
-        <v>76</v>
-      </c>
-      <c r="M39" t="s">
+      <c r="N39" t="s">
+        <v>75</v>
+      </c>
+      <c r="O39" t="s">
+        <v>76</v>
+      </c>
+      <c r="P39" t="s">
         <v>328</v>
       </c>
-      <c r="N39" t="s">
-        <v>75</v>
-      </c>
-      <c r="O39" t="s">
-        <v>76</v>
-      </c>
-      <c r="P39" t="s">
+      <c r="Q39" t="s">
+        <v>75</v>
+      </c>
+      <c r="R39" t="s">
+        <v>76</v>
+      </c>
+      <c r="S39" t="s">
+        <v>76</v>
+      </c>
+      <c r="T39" t="s">
+        <v>76</v>
+      </c>
+      <c r="U39" t="s">
+        <v>76</v>
+      </c>
+      <c r="V39" t="s">
+        <v>76</v>
+      </c>
+      <c r="W39" t="s">
+        <v>76</v>
+      </c>
+      <c r="X39" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y39" t="s">
         <v>329</v>
-      </c>
-      <c r="Q39" t="s">
-        <v>75</v>
-      </c>
-      <c r="R39" t="s">
-        <v>76</v>
-      </c>
-      <c r="S39" t="s">
-        <v>76</v>
-      </c>
-      <c r="T39" t="s">
-        <v>76</v>
-      </c>
-      <c r="U39" t="s">
-        <v>76</v>
-      </c>
-      <c r="V39" t="s">
-        <v>76</v>
-      </c>
-      <c r="W39" t="s">
-        <v>76</v>
-      </c>
-      <c r="X39" t="s">
-        <v>76</v>
-      </c>
-      <c r="Y39" t="s">
-        <v>330</v>
       </c>
       <c r="Z39" t="s">
         <v>75</v>
@@ -5039,34 +5036,34 @@
         <v>76</v>
       </c>
       <c r="G40" t="s">
+        <v>330</v>
+      </c>
+      <c r="H40" t="s">
+        <v>75</v>
+      </c>
+      <c r="I40" t="s">
+        <v>76</v>
+      </c>
+      <c r="J40" t="s">
+        <v>76</v>
+      </c>
+      <c r="K40" t="s">
+        <v>76</v>
+      </c>
+      <c r="L40" t="s">
+        <v>76</v>
+      </c>
+      <c r="M40" t="s">
         <v>331</v>
       </c>
-      <c r="H40" t="s">
-        <v>75</v>
-      </c>
-      <c r="I40" t="s">
-        <v>76</v>
-      </c>
-      <c r="J40" t="s">
-        <v>76</v>
-      </c>
-      <c r="K40" t="s">
-        <v>76</v>
-      </c>
-      <c r="L40" t="s">
-        <v>76</v>
-      </c>
-      <c r="M40" t="s">
+      <c r="N40" t="s">
+        <v>74</v>
+      </c>
+      <c r="O40" t="s">
         <v>332</v>
       </c>
-      <c r="N40" t="s">
-        <v>74</v>
-      </c>
-      <c r="O40" t="s">
+      <c r="P40" t="s">
         <v>333</v>
-      </c>
-      <c r="P40" t="s">
-        <v>334</v>
       </c>
       <c r="Q40" t="s">
         <v>74</v>
@@ -5075,7 +5072,7 @@
         <v>231</v>
       </c>
       <c r="S40" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="T40" t="s">
         <v>74</v>
@@ -5093,7 +5090,7 @@
         <v>76</v>
       </c>
       <c r="Y40" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="Z40" t="s">
         <v>75</v>
@@ -5122,25 +5119,25 @@
         <v>76</v>
       </c>
       <c r="G41" t="s">
+        <v>336</v>
+      </c>
+      <c r="H41" t="s">
+        <v>75</v>
+      </c>
+      <c r="I41" t="s">
+        <v>76</v>
+      </c>
+      <c r="J41" t="s">
         <v>337</v>
       </c>
-      <c r="H41" t="s">
-        <v>75</v>
-      </c>
-      <c r="I41" t="s">
-        <v>76</v>
-      </c>
-      <c r="J41" t="s">
+      <c r="K41" t="s">
+        <v>75</v>
+      </c>
+      <c r="L41" t="s">
+        <v>76</v>
+      </c>
+      <c r="M41" t="s">
         <v>338</v>
-      </c>
-      <c r="K41" t="s">
-        <v>75</v>
-      </c>
-      <c r="L41" t="s">
-        <v>76</v>
-      </c>
-      <c r="M41" t="s">
-        <v>339</v>
       </c>
       <c r="N41" t="s">
         <v>74</v>
@@ -5149,40 +5146,40 @@
         <v>91</v>
       </c>
       <c r="P41" t="s">
+        <v>339</v>
+      </c>
+      <c r="Q41" t="s">
+        <v>75</v>
+      </c>
+      <c r="R41" t="s">
+        <v>76</v>
+      </c>
+      <c r="S41" t="s">
+        <v>76</v>
+      </c>
+      <c r="T41" t="s">
+        <v>76</v>
+      </c>
+      <c r="U41" t="s">
+        <v>76</v>
+      </c>
+      <c r="V41" t="s">
+        <v>76</v>
+      </c>
+      <c r="W41" t="s">
+        <v>76</v>
+      </c>
+      <c r="X41" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y41" t="s">
         <v>340</v>
       </c>
-      <c r="Q41" t="s">
-        <v>75</v>
-      </c>
-      <c r="R41" t="s">
-        <v>76</v>
-      </c>
-      <c r="S41" t="s">
-        <v>76</v>
-      </c>
-      <c r="T41" t="s">
-        <v>76</v>
-      </c>
-      <c r="U41" t="s">
-        <v>76</v>
-      </c>
-      <c r="V41" t="s">
-        <v>76</v>
-      </c>
-      <c r="W41" t="s">
-        <v>76</v>
-      </c>
-      <c r="X41" t="s">
-        <v>76</v>
-      </c>
-      <c r="Y41" t="s">
+      <c r="Z41" t="s">
+        <v>74</v>
+      </c>
+      <c r="AA41" t="s">
         <v>341</v>
-      </c>
-      <c r="Z41" t="s">
-        <v>74</v>
-      </c>
-      <c r="AA41" t="s">
-        <v>342</v>
       </c>
     </row>
     <row r="42" spans="1:28" x14ac:dyDescent="0.3">
@@ -5205,7 +5202,7 @@
         <v>76</v>
       </c>
       <c r="G42" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="H42" t="s">
         <v>222</v>
@@ -5214,52 +5211,52 @@
         <v>76</v>
       </c>
       <c r="J42" t="s">
+        <v>343</v>
+      </c>
+      <c r="K42" t="s">
+        <v>75</v>
+      </c>
+      <c r="L42" t="s">
+        <v>76</v>
+      </c>
+      <c r="M42" t="s">
         <v>344</v>
       </c>
-      <c r="K42" t="s">
-        <v>75</v>
-      </c>
-      <c r="L42" t="s">
-        <v>76</v>
-      </c>
-      <c r="M42" t="s">
+      <c r="N42" t="s">
+        <v>75</v>
+      </c>
+      <c r="O42" t="s">
+        <v>76</v>
+      </c>
+      <c r="P42" t="s">
         <v>345</v>
       </c>
-      <c r="N42" t="s">
-        <v>75</v>
-      </c>
-      <c r="O42" t="s">
-        <v>76</v>
-      </c>
-      <c r="P42" t="s">
+      <c r="Q42" t="s">
+        <v>75</v>
+      </c>
+      <c r="R42" t="s">
+        <v>76</v>
+      </c>
+      <c r="S42" t="s">
         <v>346</v>
       </c>
-      <c r="Q42" t="s">
-        <v>75</v>
-      </c>
-      <c r="R42" t="s">
-        <v>76</v>
-      </c>
-      <c r="S42" t="s">
+      <c r="T42" t="s">
+        <v>75</v>
+      </c>
+      <c r="U42" t="s">
+        <v>76</v>
+      </c>
+      <c r="V42" t="s">
+        <v>76</v>
+      </c>
+      <c r="W42" t="s">
+        <v>76</v>
+      </c>
+      <c r="X42" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y42" t="s">
         <v>347</v>
-      </c>
-      <c r="T42" t="s">
-        <v>75</v>
-      </c>
-      <c r="U42" t="s">
-        <v>76</v>
-      </c>
-      <c r="V42" t="s">
-        <v>76</v>
-      </c>
-      <c r="W42" t="s">
-        <v>76</v>
-      </c>
-      <c r="X42" t="s">
-        <v>76</v>
-      </c>
-      <c r="Y42" t="s">
-        <v>348</v>
       </c>
       <c r="Z42" t="s">
         <v>75</v>
@@ -5288,61 +5285,61 @@
         <v>76</v>
       </c>
       <c r="G43" t="s">
+        <v>348</v>
+      </c>
+      <c r="H43" t="s">
+        <v>75</v>
+      </c>
+      <c r="I43" t="s">
+        <v>76</v>
+      </c>
+      <c r="J43" t="s">
         <v>349</v>
       </c>
-      <c r="H43" t="s">
-        <v>75</v>
-      </c>
-      <c r="I43" t="s">
-        <v>76</v>
-      </c>
-      <c r="J43" t="s">
+      <c r="K43" t="s">
+        <v>75</v>
+      </c>
+      <c r="L43" t="s">
+        <v>76</v>
+      </c>
+      <c r="M43" t="s">
         <v>350</v>
       </c>
-      <c r="K43" t="s">
-        <v>75</v>
-      </c>
-      <c r="L43" t="s">
-        <v>76</v>
-      </c>
-      <c r="M43" t="s">
+      <c r="N43" t="s">
+        <v>75</v>
+      </c>
+      <c r="O43" t="s">
+        <v>76</v>
+      </c>
+      <c r="P43" t="s">
         <v>351</v>
       </c>
-      <c r="N43" t="s">
-        <v>75</v>
-      </c>
-      <c r="O43" t="s">
-        <v>76</v>
-      </c>
-      <c r="P43" t="s">
+      <c r="Q43" t="s">
+        <v>75</v>
+      </c>
+      <c r="R43" t="s">
+        <v>76</v>
+      </c>
+      <c r="S43" t="s">
+        <v>76</v>
+      </c>
+      <c r="T43" t="s">
+        <v>76</v>
+      </c>
+      <c r="U43" t="s">
+        <v>76</v>
+      </c>
+      <c r="V43" t="s">
+        <v>76</v>
+      </c>
+      <c r="W43" t="s">
+        <v>76</v>
+      </c>
+      <c r="X43" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y43" t="s">
         <v>352</v>
-      </c>
-      <c r="Q43" t="s">
-        <v>75</v>
-      </c>
-      <c r="R43" t="s">
-        <v>76</v>
-      </c>
-      <c r="S43" t="s">
-        <v>76</v>
-      </c>
-      <c r="T43" t="s">
-        <v>76</v>
-      </c>
-      <c r="U43" t="s">
-        <v>76</v>
-      </c>
-      <c r="V43" t="s">
-        <v>76</v>
-      </c>
-      <c r="W43" t="s">
-        <v>76</v>
-      </c>
-      <c r="X43" t="s">
-        <v>76</v>
-      </c>
-      <c r="Y43" t="s">
-        <v>353</v>
       </c>
       <c r="Z43" t="s">
         <v>75</v>
@@ -5371,43 +5368,43 @@
         <v>76</v>
       </c>
       <c r="G44" t="s">
+        <v>353</v>
+      </c>
+      <c r="H44" t="s">
+        <v>75</v>
+      </c>
+      <c r="I44" t="s">
+        <v>76</v>
+      </c>
+      <c r="J44" t="s">
         <v>354</v>
       </c>
-      <c r="H44" t="s">
-        <v>75</v>
-      </c>
-      <c r="I44" t="s">
-        <v>76</v>
-      </c>
-      <c r="J44" t="s">
+      <c r="K44" t="s">
+        <v>75</v>
+      </c>
+      <c r="L44" t="s">
+        <v>76</v>
+      </c>
+      <c r="M44" t="s">
         <v>355</v>
       </c>
-      <c r="K44" t="s">
-        <v>75</v>
-      </c>
-      <c r="L44" t="s">
-        <v>76</v>
-      </c>
-      <c r="M44" t="s">
+      <c r="N44" t="s">
+        <v>75</v>
+      </c>
+      <c r="O44" t="s">
+        <v>76</v>
+      </c>
+      <c r="P44" t="s">
         <v>356</v>
       </c>
-      <c r="N44" t="s">
-        <v>75</v>
-      </c>
-      <c r="O44" t="s">
-        <v>76</v>
-      </c>
-      <c r="P44" t="s">
+      <c r="Q44" t="s">
+        <v>75</v>
+      </c>
+      <c r="R44" t="s">
+        <v>76</v>
+      </c>
+      <c r="S44" t="s">
         <v>357</v>
-      </c>
-      <c r="Q44" t="s">
-        <v>75</v>
-      </c>
-      <c r="R44" t="s">
-        <v>76</v>
-      </c>
-      <c r="S44" t="s">
-        <v>358</v>
       </c>
       <c r="T44" t="s">
         <v>74</v>
@@ -5425,7 +5422,7 @@
         <v>76</v>
       </c>
       <c r="Y44" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="Z44" t="s">
         <v>75</v>
@@ -5454,52 +5451,52 @@
         <v>98</v>
       </c>
       <c r="G45" t="s">
+        <v>359</v>
+      </c>
+      <c r="H45" t="s">
+        <v>75</v>
+      </c>
+      <c r="I45" t="s">
+        <v>76</v>
+      </c>
+      <c r="J45" t="s">
+        <v>76</v>
+      </c>
+      <c r="K45" t="s">
+        <v>76</v>
+      </c>
+      <c r="L45" t="s">
+        <v>76</v>
+      </c>
+      <c r="M45" t="s">
         <v>360</v>
       </c>
-      <c r="H45" t="s">
-        <v>75</v>
-      </c>
-      <c r="I45" t="s">
-        <v>76</v>
-      </c>
-      <c r="J45" t="s">
-        <v>76</v>
-      </c>
-      <c r="K45" t="s">
-        <v>76</v>
-      </c>
-      <c r="L45" t="s">
-        <v>76</v>
-      </c>
-      <c r="M45" t="s">
+      <c r="N45" t="s">
+        <v>74</v>
+      </c>
+      <c r="O45" t="s">
         <v>361</v>
       </c>
-      <c r="N45" t="s">
-        <v>74</v>
-      </c>
-      <c r="O45" t="s">
+      <c r="P45" t="s">
         <v>362</v>
       </c>
-      <c r="P45" t="s">
+      <c r="Q45" t="s">
+        <v>74</v>
+      </c>
+      <c r="R45" t="s">
         <v>363</v>
       </c>
-      <c r="Q45" t="s">
-        <v>74</v>
-      </c>
-      <c r="R45" t="s">
+      <c r="S45" t="s">
         <v>364</v>
       </c>
-      <c r="S45" t="s">
+      <c r="T45" t="s">
+        <v>75</v>
+      </c>
+      <c r="U45" t="s">
+        <v>76</v>
+      </c>
+      <c r="V45" t="s">
         <v>365</v>
-      </c>
-      <c r="T45" t="s">
-        <v>75</v>
-      </c>
-      <c r="U45" t="s">
-        <v>76</v>
-      </c>
-      <c r="V45" t="s">
-        <v>366</v>
       </c>
       <c r="W45" t="s">
         <v>74</v>
@@ -5508,7 +5505,7 @@
         <v>95</v>
       </c>
       <c r="Y45" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="Z45" t="s">
         <v>74</v>
@@ -5537,16 +5534,16 @@
         <v>76</v>
       </c>
       <c r="G46" t="s">
+        <v>367</v>
+      </c>
+      <c r="H46" t="s">
+        <v>75</v>
+      </c>
+      <c r="I46" t="s">
+        <v>76</v>
+      </c>
+      <c r="J46" t="s">
         <v>368</v>
-      </c>
-      <c r="H46" t="s">
-        <v>75</v>
-      </c>
-      <c r="I46" t="s">
-        <v>76</v>
-      </c>
-      <c r="J46" t="s">
-        <v>369</v>
       </c>
       <c r="K46" t="s">
         <v>74</v>
@@ -5555,43 +5552,43 @@
         <v>98</v>
       </c>
       <c r="M46" t="s">
+        <v>369</v>
+      </c>
+      <c r="N46" t="s">
+        <v>75</v>
+      </c>
+      <c r="O46" t="s">
+        <v>76</v>
+      </c>
+      <c r="P46" t="s">
         <v>370</v>
       </c>
-      <c r="N46" t="s">
-        <v>75</v>
-      </c>
-      <c r="O46" t="s">
-        <v>76</v>
-      </c>
-      <c r="P46" t="s">
+      <c r="Q46" t="s">
+        <v>75</v>
+      </c>
+      <c r="R46" t="s">
+        <v>76</v>
+      </c>
+      <c r="S46" t="s">
+        <v>76</v>
+      </c>
+      <c r="T46" t="s">
+        <v>76</v>
+      </c>
+      <c r="U46" t="s">
+        <v>76</v>
+      </c>
+      <c r="V46" t="s">
+        <v>76</v>
+      </c>
+      <c r="W46" t="s">
+        <v>76</v>
+      </c>
+      <c r="X46" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y46" t="s">
         <v>371</v>
-      </c>
-      <c r="Q46" t="s">
-        <v>75</v>
-      </c>
-      <c r="R46" t="s">
-        <v>76</v>
-      </c>
-      <c r="S46" t="s">
-        <v>76</v>
-      </c>
-      <c r="T46" t="s">
-        <v>76</v>
-      </c>
-      <c r="U46" t="s">
-        <v>76</v>
-      </c>
-      <c r="V46" t="s">
-        <v>76</v>
-      </c>
-      <c r="W46" t="s">
-        <v>76</v>
-      </c>
-      <c r="X46" t="s">
-        <v>76</v>
-      </c>
-      <c r="Y46" t="s">
-        <v>372</v>
       </c>
       <c r="Z46" t="s">
         <v>74</v>
@@ -5620,25 +5617,25 @@
         <v>76</v>
       </c>
       <c r="G47" t="s">
+        <v>372</v>
+      </c>
+      <c r="H47" t="s">
+        <v>75</v>
+      </c>
+      <c r="I47" t="s">
+        <v>76</v>
+      </c>
+      <c r="J47" t="s">
         <v>373</v>
       </c>
-      <c r="H47" t="s">
-        <v>75</v>
-      </c>
-      <c r="I47" t="s">
-        <v>76</v>
-      </c>
-      <c r="J47" t="s">
+      <c r="K47" t="s">
+        <v>75</v>
+      </c>
+      <c r="L47" t="s">
+        <v>76</v>
+      </c>
+      <c r="M47" t="s">
         <v>374</v>
-      </c>
-      <c r="K47" t="s">
-        <v>75</v>
-      </c>
-      <c r="L47" t="s">
-        <v>76</v>
-      </c>
-      <c r="M47" t="s">
-        <v>375</v>
       </c>
       <c r="N47" t="s">
         <v>74</v>
@@ -5647,34 +5644,34 @@
         <v>98</v>
       </c>
       <c r="P47" t="s">
+        <v>375</v>
+      </c>
+      <c r="Q47" t="s">
+        <v>75</v>
+      </c>
+      <c r="R47" t="s">
+        <v>76</v>
+      </c>
+      <c r="S47" t="s">
+        <v>76</v>
+      </c>
+      <c r="T47" t="s">
+        <v>76</v>
+      </c>
+      <c r="U47" t="s">
+        <v>76</v>
+      </c>
+      <c r="V47" t="s">
+        <v>76</v>
+      </c>
+      <c r="W47" t="s">
+        <v>76</v>
+      </c>
+      <c r="X47" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y47" t="s">
         <v>376</v>
-      </c>
-      <c r="Q47" t="s">
-        <v>75</v>
-      </c>
-      <c r="R47" t="s">
-        <v>76</v>
-      </c>
-      <c r="S47" t="s">
-        <v>76</v>
-      </c>
-      <c r="T47" t="s">
-        <v>76</v>
-      </c>
-      <c r="U47" t="s">
-        <v>76</v>
-      </c>
-      <c r="V47" t="s">
-        <v>76</v>
-      </c>
-      <c r="W47" t="s">
-        <v>76</v>
-      </c>
-      <c r="X47" t="s">
-        <v>76</v>
-      </c>
-      <c r="Y47" t="s">
-        <v>377</v>
       </c>
       <c r="Z47" t="s">
         <v>74</v>
@@ -5703,62 +5700,62 @@
         <v>76</v>
       </c>
       <c r="G48" t="s">
+        <v>377</v>
+      </c>
+      <c r="H48" t="s">
+        <v>75</v>
+      </c>
+      <c r="I48" t="s">
+        <v>76</v>
+      </c>
+      <c r="J48" t="s">
         <v>378</v>
       </c>
-      <c r="H48" t="s">
-        <v>75</v>
-      </c>
-      <c r="I48" t="s">
-        <v>76</v>
-      </c>
-      <c r="J48" t="s">
+      <c r="K48" t="s">
+        <v>75</v>
+      </c>
+      <c r="L48" t="s">
+        <v>76</v>
+      </c>
+      <c r="M48" t="s">
         <v>379</v>
       </c>
-      <c r="K48" t="s">
-        <v>75</v>
-      </c>
-      <c r="L48" t="s">
-        <v>76</v>
-      </c>
-      <c r="M48" t="s">
+      <c r="N48" t="s">
+        <v>75</v>
+      </c>
+      <c r="O48" t="s">
+        <v>76</v>
+      </c>
+      <c r="P48" t="s">
         <v>380</v>
       </c>
-      <c r="N48" t="s">
-        <v>75</v>
-      </c>
-      <c r="O48" t="s">
-        <v>76</v>
-      </c>
-      <c r="P48" t="s">
+      <c r="Q48" t="s">
+        <v>75</v>
+      </c>
+      <c r="R48" t="s">
+        <v>76</v>
+      </c>
+      <c r="S48" t="s">
         <v>381</v>
       </c>
-      <c r="Q48" t="s">
-        <v>75</v>
-      </c>
-      <c r="R48" t="s">
-        <v>76</v>
-      </c>
-      <c r="S48" t="s">
+      <c r="T48" t="s">
+        <v>75</v>
+      </c>
+      <c r="U48" t="s">
+        <v>76</v>
+      </c>
+      <c r="V48" t="s">
+        <v>76</v>
+      </c>
+      <c r="W48" t="s">
+        <v>76</v>
+      </c>
+      <c r="X48" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y48" t="s">
         <v>382</v>
       </c>
-      <c r="T48" t="s">
-        <v>75</v>
-      </c>
-      <c r="U48" t="s">
-        <v>76</v>
-      </c>
-      <c r="V48" t="s">
-        <v>76</v>
-      </c>
-      <c r="W48" t="s">
-        <v>76</v>
-      </c>
-      <c r="X48" t="s">
-        <v>76</v>
-      </c>
-      <c r="Y48" t="s">
-        <v>383</v>
-      </c>
       <c r="Z48" t="s">
         <v>75</v>
       </c>
@@ -5766,7 +5763,7 @@
         <v>76</v>
       </c>
       <c r="AB48" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="49" spans="1:27" x14ac:dyDescent="0.3">
@@ -5789,16 +5786,16 @@
         <v>76</v>
       </c>
       <c r="G49" t="s">
+        <v>383</v>
+      </c>
+      <c r="H49" t="s">
+        <v>75</v>
+      </c>
+      <c r="I49" t="s">
+        <v>76</v>
+      </c>
+      <c r="J49" t="s">
         <v>384</v>
-      </c>
-      <c r="H49" t="s">
-        <v>75</v>
-      </c>
-      <c r="I49" t="s">
-        <v>76</v>
-      </c>
-      <c r="J49" t="s">
-        <v>385</v>
       </c>
       <c r="K49" t="s">
         <v>74</v>
@@ -5807,43 +5804,43 @@
         <v>94</v>
       </c>
       <c r="M49" t="s">
+        <v>385</v>
+      </c>
+      <c r="N49" t="s">
+        <v>75</v>
+      </c>
+      <c r="O49" t="s">
+        <v>76</v>
+      </c>
+      <c r="P49" t="s">
         <v>386</v>
       </c>
-      <c r="N49" t="s">
-        <v>75</v>
-      </c>
-      <c r="O49" t="s">
-        <v>76</v>
-      </c>
-      <c r="P49" t="s">
+      <c r="Q49" t="s">
+        <v>75</v>
+      </c>
+      <c r="R49" t="s">
+        <v>76</v>
+      </c>
+      <c r="S49" t="s">
         <v>387</v>
       </c>
-      <c r="Q49" t="s">
-        <v>75</v>
-      </c>
-      <c r="R49" t="s">
-        <v>76</v>
-      </c>
-      <c r="S49" t="s">
+      <c r="T49" t="s">
+        <v>75</v>
+      </c>
+      <c r="U49" t="s">
+        <v>76</v>
+      </c>
+      <c r="V49" t="s">
+        <v>76</v>
+      </c>
+      <c r="W49" t="s">
+        <v>76</v>
+      </c>
+      <c r="X49" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y49" t="s">
         <v>388</v>
-      </c>
-      <c r="T49" t="s">
-        <v>75</v>
-      </c>
-      <c r="U49" t="s">
-        <v>76</v>
-      </c>
-      <c r="V49" t="s">
-        <v>76</v>
-      </c>
-      <c r="W49" t="s">
-        <v>76</v>
-      </c>
-      <c r="X49" t="s">
-        <v>76</v>
-      </c>
-      <c r="Y49" t="s">
-        <v>389</v>
       </c>
       <c r="Z49" t="s">
         <v>75</v>
@@ -5872,25 +5869,25 @@
         <v>76</v>
       </c>
       <c r="G50" t="s">
+        <v>389</v>
+      </c>
+      <c r="H50" t="s">
+        <v>75</v>
+      </c>
+      <c r="I50" t="s">
+        <v>76</v>
+      </c>
+      <c r="J50" t="s">
+        <v>76</v>
+      </c>
+      <c r="K50" t="s">
+        <v>76</v>
+      </c>
+      <c r="L50" t="s">
+        <v>76</v>
+      </c>
+      <c r="M50" t="s">
         <v>390</v>
-      </c>
-      <c r="H50" t="s">
-        <v>75</v>
-      </c>
-      <c r="I50" t="s">
-        <v>76</v>
-      </c>
-      <c r="J50" t="s">
-        <v>76</v>
-      </c>
-      <c r="K50" t="s">
-        <v>76</v>
-      </c>
-      <c r="L50" t="s">
-        <v>76</v>
-      </c>
-      <c r="M50" t="s">
-        <v>391</v>
       </c>
       <c r="N50" t="s">
         <v>74</v>
@@ -5899,34 +5896,34 @@
         <v>94</v>
       </c>
       <c r="P50" t="s">
+        <v>391</v>
+      </c>
+      <c r="Q50" t="s">
+        <v>75</v>
+      </c>
+      <c r="R50" t="s">
+        <v>76</v>
+      </c>
+      <c r="S50" t="s">
         <v>392</v>
       </c>
-      <c r="Q50" t="s">
-        <v>75</v>
-      </c>
-      <c r="R50" t="s">
-        <v>76</v>
-      </c>
-      <c r="S50" t="s">
+      <c r="T50" t="s">
+        <v>75</v>
+      </c>
+      <c r="U50" t="s">
+        <v>76</v>
+      </c>
+      <c r="V50" t="s">
         <v>393</v>
       </c>
-      <c r="T50" t="s">
-        <v>75</v>
-      </c>
-      <c r="U50" t="s">
-        <v>76</v>
-      </c>
-      <c r="V50" t="s">
+      <c r="W50" t="s">
+        <v>75</v>
+      </c>
+      <c r="X50" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y50" t="s">
         <v>394</v>
-      </c>
-      <c r="W50" t="s">
-        <v>75</v>
-      </c>
-      <c r="X50" t="s">
-        <v>76</v>
-      </c>
-      <c r="Y50" t="s">
-        <v>395</v>
       </c>
       <c r="Z50" t="s">
         <v>75</v>
@@ -5955,61 +5952,61 @@
         <v>76</v>
       </c>
       <c r="G51" t="s">
+        <v>395</v>
+      </c>
+      <c r="H51" t="s">
+        <v>75</v>
+      </c>
+      <c r="I51" t="s">
+        <v>76</v>
+      </c>
+      <c r="J51" t="s">
         <v>396</v>
       </c>
-      <c r="H51" t="s">
-        <v>75</v>
-      </c>
-      <c r="I51" t="s">
-        <v>76</v>
-      </c>
-      <c r="J51" t="s">
+      <c r="K51" t="s">
+        <v>75</v>
+      </c>
+      <c r="L51" t="s">
+        <v>76</v>
+      </c>
+      <c r="M51" t="s">
         <v>397</v>
       </c>
-      <c r="K51" t="s">
-        <v>75</v>
-      </c>
-      <c r="L51" t="s">
-        <v>76</v>
-      </c>
-      <c r="M51" t="s">
+      <c r="N51" t="s">
+        <v>75</v>
+      </c>
+      <c r="O51" t="s">
+        <v>76</v>
+      </c>
+      <c r="P51" t="s">
         <v>398</v>
       </c>
-      <c r="N51" t="s">
-        <v>75</v>
-      </c>
-      <c r="O51" t="s">
-        <v>76</v>
-      </c>
-      <c r="P51" t="s">
+      <c r="Q51" t="s">
+        <v>75</v>
+      </c>
+      <c r="R51" t="s">
+        <v>76</v>
+      </c>
+      <c r="S51" t="s">
+        <v>76</v>
+      </c>
+      <c r="T51" t="s">
+        <v>76</v>
+      </c>
+      <c r="U51" t="s">
+        <v>76</v>
+      </c>
+      <c r="V51" t="s">
+        <v>76</v>
+      </c>
+      <c r="W51" t="s">
+        <v>76</v>
+      </c>
+      <c r="X51" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y51" t="s">
         <v>399</v>
-      </c>
-      <c r="Q51" t="s">
-        <v>75</v>
-      </c>
-      <c r="R51" t="s">
-        <v>76</v>
-      </c>
-      <c r="S51" t="s">
-        <v>76</v>
-      </c>
-      <c r="T51" t="s">
-        <v>76</v>
-      </c>
-      <c r="U51" t="s">
-        <v>76</v>
-      </c>
-      <c r="V51" t="s">
-        <v>76</v>
-      </c>
-      <c r="W51" t="s">
-        <v>76</v>
-      </c>
-      <c r="X51" t="s">
-        <v>76</v>
-      </c>
-      <c r="Y51" t="s">
-        <v>400</v>
       </c>
       <c r="Z51" t="s">
         <v>75</v>
@@ -6023,76 +6020,76 @@
         <v>20</v>
       </c>
       <c r="B52" t="s">
+        <v>400</v>
+      </c>
+      <c r="C52" t="s">
+        <v>76</v>
+      </c>
+      <c r="D52" t="s">
+        <v>76</v>
+      </c>
+      <c r="E52" t="s">
+        <v>75</v>
+      </c>
+      <c r="F52" t="s">
+        <v>76</v>
+      </c>
+      <c r="G52" t="s">
         <v>401</v>
       </c>
-      <c r="C52" t="s">
-        <v>76</v>
-      </c>
-      <c r="D52" t="s">
-        <v>76</v>
-      </c>
-      <c r="E52" t="s">
-        <v>75</v>
-      </c>
-      <c r="F52" t="s">
-        <v>76</v>
-      </c>
-      <c r="G52" t="s">
+      <c r="H52" t="s">
+        <v>75</v>
+      </c>
+      <c r="I52" t="s">
+        <v>76</v>
+      </c>
+      <c r="J52" t="s">
+        <v>76</v>
+      </c>
+      <c r="K52" t="s">
+        <v>76</v>
+      </c>
+      <c r="L52" t="s">
+        <v>76</v>
+      </c>
+      <c r="M52" t="s">
         <v>402</v>
       </c>
-      <c r="H52" t="s">
-        <v>75</v>
-      </c>
-      <c r="I52" t="s">
-        <v>76</v>
-      </c>
-      <c r="J52" t="s">
-        <v>76</v>
-      </c>
-      <c r="K52" t="s">
-        <v>76</v>
-      </c>
-      <c r="L52" t="s">
-        <v>76</v>
-      </c>
-      <c r="M52" t="s">
+      <c r="N52" t="s">
+        <v>75</v>
+      </c>
+      <c r="O52" t="s">
+        <v>76</v>
+      </c>
+      <c r="P52" t="s">
         <v>403</v>
       </c>
-      <c r="N52" t="s">
-        <v>75</v>
-      </c>
-      <c r="O52" t="s">
-        <v>76</v>
-      </c>
-      <c r="P52" t="s">
+      <c r="Q52" t="s">
+        <v>75</v>
+      </c>
+      <c r="R52" t="s">
+        <v>76</v>
+      </c>
+      <c r="S52" t="s">
         <v>404</v>
       </c>
-      <c r="Q52" t="s">
-        <v>75</v>
-      </c>
-      <c r="R52" t="s">
-        <v>76</v>
-      </c>
-      <c r="S52" t="s">
+      <c r="T52" t="s">
+        <v>75</v>
+      </c>
+      <c r="U52" t="s">
+        <v>76</v>
+      </c>
+      <c r="V52" t="s">
+        <v>76</v>
+      </c>
+      <c r="W52" t="s">
+        <v>76</v>
+      </c>
+      <c r="X52" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y52" t="s">
         <v>405</v>
-      </c>
-      <c r="T52" t="s">
-        <v>75</v>
-      </c>
-      <c r="U52" t="s">
-        <v>76</v>
-      </c>
-      <c r="V52" t="s">
-        <v>76</v>
-      </c>
-      <c r="W52" t="s">
-        <v>76</v>
-      </c>
-      <c r="X52" t="s">
-        <v>76</v>
-      </c>
-      <c r="Y52" t="s">
-        <v>406</v>
       </c>
       <c r="Z52" t="s">
         <v>75</v>
@@ -6121,43 +6118,43 @@
         <v>76</v>
       </c>
       <c r="G53" t="s">
+        <v>406</v>
+      </c>
+      <c r="H53" t="s">
+        <v>75</v>
+      </c>
+      <c r="I53" t="s">
+        <v>76</v>
+      </c>
+      <c r="J53" t="s">
+        <v>76</v>
+      </c>
+      <c r="K53" t="s">
+        <v>76</v>
+      </c>
+      <c r="L53" t="s">
+        <v>76</v>
+      </c>
+      <c r="M53" t="s">
         <v>407</v>
       </c>
-      <c r="H53" t="s">
-        <v>75</v>
-      </c>
-      <c r="I53" t="s">
-        <v>76</v>
-      </c>
-      <c r="J53" t="s">
-        <v>76</v>
-      </c>
-      <c r="K53" t="s">
-        <v>76</v>
-      </c>
-      <c r="L53" t="s">
-        <v>76</v>
-      </c>
-      <c r="M53" t="s">
+      <c r="N53" t="s">
+        <v>74</v>
+      </c>
+      <c r="O53" t="s">
         <v>408</v>
       </c>
-      <c r="N53" t="s">
-        <v>74</v>
-      </c>
-      <c r="O53" t="s">
+      <c r="P53" t="s">
         <v>409</v>
       </c>
-      <c r="P53" t="s">
+      <c r="Q53" t="s">
+        <v>75</v>
+      </c>
+      <c r="R53" t="s">
+        <v>76</v>
+      </c>
+      <c r="S53" t="s">
         <v>410</v>
-      </c>
-      <c r="Q53" t="s">
-        <v>75</v>
-      </c>
-      <c r="R53" t="s">
-        <v>76</v>
-      </c>
-      <c r="S53" t="s">
-        <v>411</v>
       </c>
       <c r="T53" t="s">
         <v>74</v>
@@ -6166,7 +6163,7 @@
         <v>91</v>
       </c>
       <c r="V53" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="W53" t="s">
         <v>74</v>
@@ -6175,7 +6172,7 @@
         <v>92</v>
       </c>
       <c r="Y53" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="Z53" t="s">
         <v>75</v>
@@ -6204,61 +6201,61 @@
         <v>76</v>
       </c>
       <c r="G54" t="s">
+        <v>413</v>
+      </c>
+      <c r="H54" t="s">
+        <v>75</v>
+      </c>
+      <c r="I54" t="s">
+        <v>76</v>
+      </c>
+      <c r="J54" t="s">
         <v>414</v>
       </c>
-      <c r="H54" t="s">
-        <v>75</v>
-      </c>
-      <c r="I54" t="s">
-        <v>76</v>
-      </c>
-      <c r="J54" t="s">
+      <c r="K54" t="s">
+        <v>75</v>
+      </c>
+      <c r="L54" t="s">
+        <v>76</v>
+      </c>
+      <c r="M54" t="s">
         <v>415</v>
       </c>
-      <c r="K54" t="s">
-        <v>75</v>
-      </c>
-      <c r="L54" t="s">
-        <v>76</v>
-      </c>
-      <c r="M54" t="s">
+      <c r="N54" t="s">
+        <v>75</v>
+      </c>
+      <c r="O54" t="s">
+        <v>76</v>
+      </c>
+      <c r="P54" t="s">
         <v>416</v>
       </c>
-      <c r="N54" t="s">
-        <v>75</v>
-      </c>
-      <c r="O54" t="s">
-        <v>76</v>
-      </c>
-      <c r="P54" t="s">
+      <c r="Q54" t="s">
+        <v>75</v>
+      </c>
+      <c r="R54" t="s">
+        <v>76</v>
+      </c>
+      <c r="S54" t="s">
         <v>417</v>
       </c>
-      <c r="Q54" t="s">
-        <v>75</v>
-      </c>
-      <c r="R54" t="s">
-        <v>76</v>
-      </c>
-      <c r="S54" t="s">
+      <c r="T54" t="s">
+        <v>75</v>
+      </c>
+      <c r="U54" t="s">
+        <v>76</v>
+      </c>
+      <c r="V54" t="s">
         <v>418</v>
       </c>
-      <c r="T54" t="s">
-        <v>75</v>
-      </c>
-      <c r="U54" t="s">
-        <v>76</v>
-      </c>
-      <c r="V54" t="s">
+      <c r="W54" t="s">
+        <v>75</v>
+      </c>
+      <c r="X54" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y54" t="s">
         <v>419</v>
-      </c>
-      <c r="W54" t="s">
-        <v>75</v>
-      </c>
-      <c r="X54" t="s">
-        <v>76</v>
-      </c>
-      <c r="Y54" t="s">
-        <v>420</v>
       </c>
       <c r="Z54" t="s">
         <v>75</v>

</xml_diff>